<commit_message>
Add private user accounts, notes API and PostgreSQL deployment support
</commit_message>
<xml_diff>
--- a/sample_docs/ac_warranty.xlsx
+++ b/sample_docs/ac_warranty.xlsx
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46180</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="5">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46910</v>
+        <v>46920</v>
       </c>
     </row>
     <row r="6">

</xml_diff>